<commit_message>
style(premissas): vírgula decimal nas notas de origem e taxa única dita com clareza
As notas que aparecem na planilha e na página traziam percentuais com ponto
(12.2% a 15.3%). A nota do custo da dívida passa a dizer que a taxa do
Tesouro de dez anos é a mesma para as três empresas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015bsZAfNcZxGVdaRRin3Zom
</commit_message>
<xml_diff>
--- a/saida/valuation_vale_csn_gerdau.xlsx
+++ b/saida/valuation_vale_csn_gerdau.xlsx
@@ -2233,13 +2233,13 @@
     <t xml:space="preserve">De onde veio</t>
   </si>
   <si>
-    <t xml:space="preserve">2026: nível dos últimos 12 meses (LTM 2T26). Pessimista: receita parada, ou seja, queda real. Moderado: inflação esperada no Focus para 2027-2030, crescimento real zero. Otimista: crescimento médio da receita de 2018 a 2025 (6.8% ao ano).</t>
+    <t xml:space="preserve">2026: nível dos últimos 12 meses (LTM 2T26). Pessimista: receita parada, ou seja, queda real. Moderado: inflação esperada no Focus para 2027-2030, crescimento real zero. Otimista: crescimento médio da receita de 2018 a 2025 (6,8% ao ano).</t>
   </si>
   <si>
     <t xml:space="preserve">2026: nível dos últimos 12 meses (LTM 2T26). Daí até 2030 em linha reta. Faixa: margem EBITDA de 2021 a 2025, sem perdas por recuperabilidade. Pessimista é o segundo pior ano, moderado a mediana e otimista o segundo melhor.</t>
   </si>
   <si>
-    <t xml:space="preserve">Moderado: o WACC que sai do CAPM. O juro prefixado longo andou de 12.2% a 15.3% nos últimos dois anos; pessimista e otimista deslocam o WACC em metade dessa amplitude.</t>
+    <t xml:space="preserve">Moderado: o WACC que sai do CAPM. O juro prefixado longo andou de 12,2% a 15,3% nos últimos dois anos; pessimista e otimista deslocam o WACC em metade dessa amplitude.</t>
   </si>
   <si>
     <t xml:space="preserve">Vendas, administrativas e outras, sem perdas por recuperabilidade. Do nível dos últimos 12 meses até a mediana de 2021-2025.</t>
@@ -2260,7 +2260,7 @@
     <t xml:space="preserve">Alíquota nominal: IRPJ 25% + CSLL 9%.</t>
   </si>
   <si>
-    <t xml:space="preserve">Piso: a taxa do Tesouro prefixado de dez anos, sem spread de crédito. Custo implícito mediano 2023-2025: 17.8%.</t>
+    <t xml:space="preserve">A taxa do Tesouro prefixado de dez anos, a mesma para as três empresas. Custo implícito mediano 2023-2025: 17,8%.</t>
   </si>
   <si>
     <t xml:space="preserve">Mediana 2023-2025 da receita financeira sobre o caixa médio.</t>
@@ -2272,7 +2272,7 @@
     <t xml:space="preserve">Tesouro prefixado de dez anos (em reais, nominal).</t>
   </si>
   <si>
-    <t xml:space="preserve">Regressão de 5 anos, retornos semanais contra o BOVA11, preços sem ajuste de proventos. Beta de 2 anos: 0.64.</t>
+    <t xml:space="preserve">Regressão de 5 anos, retornos semanais contra o BOVA11, preços sem ajuste de proventos. Beta de 2 anos: 0,64.</t>
   </si>
   <si>
     <t xml:space="preserve">Damodaran, mercado maduro. O risco-país já está no juro em reais.</t>
@@ -2311,22 +2311,22 @@
     <t xml:space="preserve">Pregão do preço acima.</t>
   </si>
   <si>
-    <t xml:space="preserve">2026: nível dos últimos 12 meses (LTM 2T26). Pessimista: receita parada, ou seja, queda real. Moderado: inflação esperada no Focus para 2027-2030, crescimento real zero. Otimista: crescimento médio da receita de 2018 a 2025 (10.0% ao ano), limitado a 4% acima da inflação porque parte veio de aquisições.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Piso: a taxa do Tesouro prefixado de dez anos, sem spread de crédito. Custo implícito mediano 2023-2025: 14.2%.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regressão de 5 anos, retornos semanais contra o BOVA11, preços sem ajuste de proventos. Beta de 2 anos: 1.48.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026: nível dos últimos 12 meses (LTM 2T26). Pessimista: receita parada, ou seja, queda real. Moderado: inflação esperada no Focus para 2027-2030, crescimento real zero. Otimista: crescimento médio da receita de 2018 a 2025 (6.1% ao ano).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Piso: a taxa do Tesouro prefixado de dez anos, sem spread de crédito. Custo implícito mediano 2023-2025: 19.3%.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regressão de 5 anos, retornos semanais contra o BOVA11, preços sem ajuste de proventos. Beta de 2 anos: 0.71.</t>
+    <t xml:space="preserve">2026: nível dos últimos 12 meses (LTM 2T26). Pessimista: receita parada, ou seja, queda real. Moderado: inflação esperada no Focus para 2027-2030, crescimento real zero. Otimista: crescimento médio da receita de 2018 a 2025 (10,0% ao ano), limitado a 4% acima da inflação porque parte veio de aquisições.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A taxa do Tesouro prefixado de dez anos, a mesma para as três empresas. Custo implícito mediano 2023-2025: 14,2%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regressão de 5 anos, retornos semanais contra o BOVA11, preços sem ajuste de proventos. Beta de 2 anos: 1,48.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026: nível dos últimos 12 meses (LTM 2T26). Pessimista: receita parada, ou seja, queda real. Moderado: inflação esperada no Focus para 2027-2030, crescimento real zero. Otimista: crescimento médio da receita de 2018 a 2025 (6,1% ao ano).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A taxa do Tesouro prefixado de dez anos, a mesma para as três empresas. Custo implícito mediano 2023-2025: 19,3%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regressão de 5 anos, retornos semanais contra o BOVA11, preços sem ajuste de proventos. Beta de 2 anos: 0,71.</t>
   </si>
   <si>
     <t xml:space="preserve">Dados da CVM</t>
@@ -2986,11 +2986,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="382606"/>
-        <c:axId val="86157532"/>
+        <c:axId val="65242280"/>
+        <c:axId val="71378906"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="382606"/>
+        <c:axId val="65242280"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3022,7 +3022,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86157532"/>
+        <c:crossAx val="71378906"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3030,7 +3030,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="86157532"/>
+        <c:axId val="71378906"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3072,7 +3072,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="382606"/>
+        <c:crossAx val="65242280"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4124,11 +4124,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="58037023"/>
-        <c:axId val="28988576"/>
+        <c:axId val="80750784"/>
+        <c:axId val="97798197"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="58037023"/>
+        <c:axId val="80750784"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4160,7 +4160,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="28988576"/>
+        <c:crossAx val="97798197"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4168,7 +4168,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="28988576"/>
+        <c:axId val="97798197"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4210,7 +4210,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58037023"/>
+        <c:crossAx val="80750784"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4790,11 +4790,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="94622550"/>
-        <c:axId val="19950160"/>
+        <c:axId val="3846684"/>
+        <c:axId val="90065978"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="94622550"/>
+        <c:axId val="3846684"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4836,12 +4836,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19950160"/>
+        <c:crossAx val="90065978"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="19950160"/>
+        <c:axId val="90065978"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4883,7 +4883,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94622550"/>
+        <c:crossAx val="3846684"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>

</xml_diff>

<commit_message>
docs(planilha, registro): aviso de que não é recomendação, nas palavras do autor
O Painel da planilha e a fotografia do dia deixam de falar em proposta ainda
não revisada e passam a dizer o que o estudo é: uma análise com os dados que
as empresas divulgam e simulações com dados reais e projetados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015bsZAfNcZxGVdaRRin3Zom
</commit_message>
<xml_diff>
--- a/saida/valuation_vale_csn_gerdau.xlsx
+++ b/saida/valuation_vale_csn_gerdau.xlsx
@@ -40,7 +40,7 @@
     <t xml:space="preserve">Escolha a empresa e o cenário nas células amarelas. Todas as abas recalculam.</t>
   </si>
   <si>
-    <t xml:space="preserve">Estudo acadêmico e de portfólio, com dados públicos da CVM e da B3. Não é recomendação de compra ou venda. As premissas são uma proposta por regra, ainda não revisada.</t>
+    <t xml:space="preserve">Isto não é recomendação de investimento. É uma análise feita com os dados que as próprias empresas divulgam e com simulações que juntam dados reais e dados projetados.</t>
   </si>
   <si>
     <t xml:space="preserve">Listas (não apagar)</t>
@@ -2986,11 +2986,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="65242280"/>
-        <c:axId val="71378906"/>
+        <c:axId val="56982360"/>
+        <c:axId val="45477913"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="65242280"/>
+        <c:axId val="56982360"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3022,7 +3022,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71378906"/>
+        <c:crossAx val="45477913"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3030,7 +3030,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="71378906"/>
+        <c:axId val="45477913"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3072,7 +3072,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65242280"/>
+        <c:crossAx val="56982360"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4124,11 +4124,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="80750784"/>
-        <c:axId val="97798197"/>
+        <c:axId val="2944039"/>
+        <c:axId val="25292030"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="80750784"/>
+        <c:axId val="2944039"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4160,7 +4160,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97798197"/>
+        <c:crossAx val="25292030"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4168,7 +4168,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="97798197"/>
+        <c:axId val="25292030"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4210,7 +4210,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80750784"/>
+        <c:crossAx val="2944039"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4790,11 +4790,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="3846684"/>
-        <c:axId val="90065978"/>
+        <c:axId val="94474264"/>
+        <c:axId val="92860748"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="3846684"/>
+        <c:axId val="94474264"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4836,12 +4836,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="90065978"/>
+        <c:crossAx val="92860748"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="90065978"/>
+        <c:axId val="92860748"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4883,7 +4883,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="3846684"/>
+        <c:crossAx val="94474264"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>

</xml_diff>